<commit_message>
them nut nhap thu cong
</commit_message>
<xml_diff>
--- a/samples/bang-cong-mau.xlsx
+++ b/samples/bang-cong-mau.xlsx
@@ -1,26 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DoANJava\QuanLyLuong\samples\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DuLieuDaiHoc\2026nam3\KI-2\ontap-jva\QuanLyLuong\samples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB8DC56A-83D4-48C6-A68D-A7C8372DED80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD6E6CB1-9226-481E-87CE-53ADC6AD9A3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BangCongMau" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>employeeCode</t>
   </si>
@@ -55,55 +60,7 @@
     <t>note</t>
   </si>
   <si>
-    <t>EMP0003</t>
-  </si>
-  <si>
-    <t>2026-03-01</t>
-  </si>
-  <si>
-    <t>08:00</t>
-  </si>
-  <si>
-    <t>17:30</t>
-  </si>
-  <si>
-    <t>MAY-01</t>
-  </si>
-  <si>
-    <t>Ca ngay</t>
-  </si>
-  <si>
-    <t>EMP0002</t>
-  </si>
-  <si>
-    <t>2026-03-02</t>
-  </si>
-  <si>
-    <t>08:15</t>
-  </si>
-  <si>
     <t>17:00</t>
-  </si>
-  <si>
-    <t>Di tre 15p</t>
-  </si>
-  <si>
-    <t>EMP0004</t>
-  </si>
-  <si>
-    <t>2026-03-09</t>
-  </si>
-  <si>
-    <t>18:00</t>
-  </si>
-  <si>
-    <t>MAY-02</t>
-  </si>
-  <si>
-    <t>Tang ca ngay thuong</t>
-  </si>
-  <si>
-    <t>EMP0001</t>
   </si>
   <si>
     <t>2026-03-20</t>
@@ -488,22 +445,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="23" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="23.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -538,9 +495,9 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s">
         <v>12</v>
@@ -549,168 +506,28 @@
         <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E2">
         <v>8</v>
       </c>
       <c r="F2">
-        <v>1.5</v>
+        <v>0</v>
       </c>
       <c r="G2">
         <v>0</v>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I2">
         <v>0</v>
       </c>
       <c r="J2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K2" t="s">
         <v>15</v>
-      </c>
-      <c r="K2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" t="s">
-        <v>19</v>
-      </c>
-      <c r="D3" t="s">
-        <v>20</v>
-      </c>
-      <c r="E3">
-        <v>7.75</v>
-      </c>
-      <c r="F3">
-        <v>0</v>
-      </c>
-      <c r="G3">
-        <v>0</v>
-      </c>
-      <c r="H3">
-        <v>0</v>
-      </c>
-      <c r="I3">
-        <v>15</v>
-      </c>
-      <c r="J3" t="s">
-        <v>15</v>
-      </c>
-      <c r="K3" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" t="s">
-        <v>24</v>
-      </c>
-      <c r="E4">
-        <v>8</v>
-      </c>
-      <c r="F4">
-        <v>2</v>
-      </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-      <c r="H4">
-        <v>0</v>
-      </c>
-      <c r="I4">
-        <v>0</v>
-      </c>
-      <c r="J4" t="s">
-        <v>25</v>
-      </c>
-      <c r="K4" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B5" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" t="s">
-        <v>29</v>
-      </c>
-      <c r="D5" t="s">
-        <v>20</v>
-      </c>
-      <c r="E5">
-        <v>8</v>
-      </c>
-      <c r="F5">
-        <v>0</v>
-      </c>
-      <c r="G5">
-        <v>0</v>
-      </c>
-      <c r="H5">
-        <v>2</v>
-      </c>
-      <c r="I5">
-        <v>0</v>
-      </c>
-      <c r="J5" t="s">
-        <v>30</v>
-      </c>
-      <c r="K5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>32</v>
-      </c>
-      <c r="B6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C6" t="s">
-        <v>29</v>
-      </c>
-      <c r="D6" t="s">
-        <v>20</v>
-      </c>
-      <c r="E6">
-        <v>8</v>
-      </c>
-      <c r="F6">
-        <v>0</v>
-      </c>
-      <c r="G6">
-        <v>0</v>
-      </c>
-      <c r="H6">
-        <v>2</v>
-      </c>
-      <c r="I6">
-        <v>0</v>
-      </c>
-      <c r="J6" t="s">
-        <v>30</v>
-      </c>
-      <c r="K6" t="s">
-        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>